<commit_message>
fixbug/fsel-4664_fsel-6010: Update Export file Report Learning Result
</commit_message>
<xml_diff>
--- a/Services/Fsel.Course/Fsel.Course.Lms.Api/Resources/ManagerReports/BaoCaoKetQuaHocTapEF.xlsx
+++ b/Services/Fsel.Course/Fsel.Course.Lms.Api/Resources/ManagerReports/BaoCaoKetQuaHocTapEF.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Work\Backend\fsel_src\Services\Fsel.Course\Fsel.Course.Lms.Api\Resources\ManagerReports\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\PhanPhuc\Fsel\fsel_src\Services\Fsel.Course\Fsel.Course.Lms.Api\Resources\ManagerReports\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{988435F6-CC14-4EBB-A317-08BB0B18669F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6F05BAB5-1E5F-42AC-8B91-F14C3E7ADBE3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{A3E0742E-2868-4C52-ABF9-706A4D9673F5}"/>
+    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{A3E0742E-2868-4C52-ABF9-706A4D9673F5}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="56" uniqueCount="55">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="67" uniqueCount="56">
   <si>
     <t>Trường</t>
   </si>
@@ -144,9 +144,6 @@
     <t>Unit 12 : {0}</t>
   </si>
   <si>
-    <t>{0}</t>
-  </si>
-  <si>
     <t>Trạng thái: {0}</t>
   </si>
   <si>
@@ -190,6 +187,12 @@
   </si>
   <si>
     <t>Điểm tổng trung bình: {0}</t>
+  </si>
+  <si>
+    <t>0 hs</t>
+  </si>
+  <si>
+    <t>[SchoolName]</t>
   </si>
 </sst>
 </file>
@@ -347,16 +350,13 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="19">
+  <cellXfs count="18">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
@@ -379,10 +379,10 @@
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
+      <alignment horizontal="left" wrapText="1"/>
     </xf>
     <xf numFmtId="9" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
+      <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left"/>
@@ -718,13 +718,14 @@
   <cols>
     <col min="1" max="1" width="20.875" customWidth="1"/>
     <col min="2" max="3" width="28.875" customWidth="1"/>
-    <col min="7" max="7" width="14.5" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="23.125" customWidth="1"/>
-    <col min="9" max="9" width="19.75" customWidth="1"/>
-    <col min="10" max="10" width="19.5" customWidth="1"/>
-    <col min="11" max="11" width="17.5" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="27.125" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="18" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="15.375" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="22.625" customWidth="1"/>
+    <col min="8" max="8" width="18.25" customWidth="1"/>
+    <col min="9" max="9" width="16.25" customWidth="1"/>
+    <col min="10" max="10" width="14.875" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="30.5" customWidth="1"/>
+    <col min="12" max="12" width="22.75" customWidth="1"/>
+    <col min="13" max="13" width="15.5" customWidth="1"/>
     <col min="14" max="14" width="18.125" bestFit="1" customWidth="1"/>
     <col min="15" max="15" width="17" customWidth="1"/>
     <col min="16" max="16" width="18.25" customWidth="1"/>
@@ -738,50 +739,52 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:24" ht="26.25" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A1" s="16" t="s">
+      <c r="A1" s="15" t="s">
         <v>26</v>
       </c>
-      <c r="B1" s="17"/>
-      <c r="C1" s="17"/>
-      <c r="D1" s="17"/>
-      <c r="E1" s="17"/>
-      <c r="F1" s="17"/>
-      <c r="G1" s="17"/>
-      <c r="H1" s="17"/>
-      <c r="I1" s="17"/>
-      <c r="J1" s="17"/>
-      <c r="K1" s="17"/>
-      <c r="L1" s="17"/>
-      <c r="M1" s="17"/>
-      <c r="N1" s="17"/>
-      <c r="O1" s="17"/>
-      <c r="P1" s="17"/>
-      <c r="Q1" s="17"/>
-      <c r="R1" s="17"/>
-      <c r="S1" s="17"/>
-      <c r="T1" s="17"/>
-      <c r="U1" s="17"/>
-      <c r="V1" s="17"/>
-      <c r="W1" s="17"/>
-      <c r="X1" s="17"/>
+      <c r="B1" s="16"/>
+      <c r="C1" s="16"/>
+      <c r="D1" s="16"/>
+      <c r="E1" s="16"/>
+      <c r="F1" s="16"/>
+      <c r="G1" s="16"/>
+      <c r="H1" s="16"/>
+      <c r="I1" s="16"/>
+      <c r="J1" s="16"/>
+      <c r="K1" s="16"/>
+      <c r="L1" s="16"/>
+      <c r="M1" s="16"/>
+      <c r="N1" s="16"/>
+      <c r="O1" s="16"/>
+      <c r="P1" s="16"/>
+      <c r="Q1" s="16"/>
+      <c r="R1" s="16"/>
+      <c r="S1" s="16"/>
+      <c r="T1" s="16"/>
+      <c r="U1" s="16"/>
+      <c r="V1" s="16"/>
+      <c r="W1" s="16"/>
+      <c r="X1" s="16"/>
     </row>
-    <row r="2" spans="1:24" s="10" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A2" s="18" t="s">
+    <row r="2" spans="1:24" s="9" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A2" s="17" t="s">
         <v>0</v>
       </c>
-      <c r="B2" s="18"/>
-      <c r="C2" s="18"/>
-      <c r="D2" s="18"/>
-      <c r="E2" s="18"/>
-      <c r="F2" s="18"/>
-      <c r="G2" s="2" t="s">
+      <c r="B2" s="17"/>
+      <c r="C2" s="17"/>
+      <c r="D2" s="17"/>
+      <c r="E2" s="17"/>
+      <c r="F2" s="1" t="s">
+        <v>55</v>
+      </c>
+      <c r="G2" s="1" t="s">
         <v>39</v>
       </c>
       <c r="H2" s="1" t="s">
         <v>40</v>
       </c>
       <c r="I2" s="1" t="s">
-        <v>41</v>
+        <v>51</v>
       </c>
       <c r="J2" s="1" t="s">
         <v>52</v>
@@ -790,327 +793,337 @@
         <v>53</v>
       </c>
       <c r="L2" s="1" t="s">
-        <v>54</v>
+        <v>41</v>
       </c>
       <c r="M2" s="1" t="s">
         <v>42</v>
       </c>
-      <c r="N2" s="1" t="s">
+      <c r="N2" s="3"/>
+      <c r="O2" s="3"/>
+      <c r="P2" s="10"/>
+      <c r="Q2" s="10"/>
+      <c r="R2" s="10"/>
+      <c r="S2" s="10"/>
+      <c r="T2" s="10"/>
+      <c r="U2" s="10"/>
+      <c r="V2" s="10"/>
+      <c r="W2" s="10"/>
+      <c r="X2" s="10"/>
+    </row>
+    <row r="3" spans="1:24" s="9" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A3" s="13" t="s">
+        <v>1</v>
+      </c>
+      <c r="B3" s="13"/>
+      <c r="C3" s="13"/>
+      <c r="D3" s="13"/>
+      <c r="E3" s="13"/>
+      <c r="F3" s="1">
+        <v>0</v>
+      </c>
+      <c r="G3" s="2"/>
+      <c r="H3" s="3"/>
+      <c r="I3" s="3"/>
+      <c r="J3" s="3"/>
+      <c r="K3" s="3"/>
+      <c r="L3" s="3"/>
+      <c r="M3" s="3"/>
+      <c r="N3" s="10"/>
+      <c r="O3" s="10"/>
+      <c r="P3" s="10"/>
+      <c r="Q3" s="10"/>
+      <c r="R3" s="10"/>
+      <c r="S3" s="10"/>
+      <c r="T3" s="10"/>
+      <c r="U3" s="10"/>
+      <c r="V3" s="10"/>
+      <c r="W3" s="10"/>
+      <c r="X3" s="10"/>
+    </row>
+    <row r="4" spans="1:24" s="9" customFormat="1" ht="30.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A4" s="13" t="s">
+        <v>2</v>
+      </c>
+      <c r="B4" s="13"/>
+      <c r="C4" s="13"/>
+      <c r="D4" s="13"/>
+      <c r="E4" s="13"/>
+      <c r="F4" s="1" t="s">
         <v>43</v>
       </c>
-      <c r="O2" s="4"/>
-      <c r="P2" s="4" t="s">
-        <v>43</v>
-      </c>
-      <c r="Q2" s="11"/>
-      <c r="R2" s="11"/>
-      <c r="S2" s="11"/>
-      <c r="T2" s="11"/>
-      <c r="U2" s="11"/>
-      <c r="V2" s="11"/>
-      <c r="W2" s="11"/>
-      <c r="X2" s="11"/>
-    </row>
-    <row r="3" spans="1:24" s="10" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A3" s="14" t="s">
-        <v>1</v>
-      </c>
-      <c r="B3" s="14"/>
-      <c r="C3" s="14"/>
-      <c r="D3" s="14"/>
-      <c r="E3" s="14"/>
-      <c r="F3" s="14"/>
-      <c r="G3" s="2">
-        <v>0</v>
-      </c>
-      <c r="H3" s="2"/>
-      <c r="I3" s="4"/>
-      <c r="J3" s="4"/>
-      <c r="K3" s="4"/>
-      <c r="L3" s="4"/>
-      <c r="M3" s="4"/>
-      <c r="N3" s="4"/>
-      <c r="O3" s="11"/>
-      <c r="P3" s="11"/>
-      <c r="Q3" s="11"/>
-      <c r="R3" s="11"/>
-      <c r="S3" s="11"/>
-      <c r="T3" s="11"/>
-      <c r="U3" s="11"/>
-      <c r="V3" s="11"/>
-      <c r="W3" s="11"/>
-      <c r="X3" s="11"/>
-    </row>
-    <row r="4" spans="1:24" s="10" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A4" s="14" t="s">
-        <v>2</v>
-      </c>
-      <c r="B4" s="14"/>
-      <c r="C4" s="14"/>
-      <c r="D4" s="14"/>
-      <c r="E4" s="14"/>
-      <c r="F4" s="14"/>
-      <c r="G4" s="2" t="s">
+      <c r="G4" s="1" t="s">
         <v>44</v>
       </c>
-      <c r="H4" s="2" t="s">
+      <c r="H4" s="1" t="s">
         <v>45</v>
       </c>
-      <c r="I4" s="2" t="s">
-        <v>46</v>
-      </c>
+      <c r="I4" s="2"/>
       <c r="J4" s="2"/>
       <c r="K4" s="2"/>
-      <c r="L4" s="2"/>
-      <c r="M4" s="4"/>
-      <c r="N4" s="4"/>
-      <c r="O4" s="11"/>
-      <c r="P4" s="11"/>
-      <c r="Q4" s="11"/>
-      <c r="R4" s="11"/>
-      <c r="S4" s="11"/>
-      <c r="T4" s="11"/>
-      <c r="U4" s="11"/>
-      <c r="V4" s="11"/>
-      <c r="W4" s="11"/>
-      <c r="X4" s="11"/>
+      <c r="L4" s="3"/>
+      <c r="M4" s="3"/>
+      <c r="N4" s="10"/>
+      <c r="O4" s="10"/>
+      <c r="P4" s="10"/>
+      <c r="Q4" s="10"/>
+      <c r="R4" s="10"/>
+      <c r="S4" s="10"/>
+      <c r="T4" s="10"/>
+      <c r="U4" s="10"/>
+      <c r="V4" s="10"/>
+      <c r="W4" s="10"/>
+      <c r="X4" s="10"/>
     </row>
-    <row r="5" spans="1:24" s="10" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A5" s="14" t="s">
+    <row r="5" spans="1:24" s="9" customFormat="1" ht="24.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A5" s="13" t="s">
+        <v>49</v>
+      </c>
+      <c r="B5" s="13"/>
+      <c r="C5" s="13"/>
+      <c r="D5" s="13"/>
+      <c r="E5" s="13"/>
+      <c r="F5" s="1" t="s">
         <v>50</v>
       </c>
-      <c r="B5" s="14"/>
-      <c r="C5" s="14"/>
-      <c r="D5" s="14"/>
-      <c r="E5" s="14"/>
-      <c r="F5" s="14"/>
-      <c r="G5" s="1" t="s">
-        <v>51</v>
-      </c>
+      <c r="G5" s="1"/>
       <c r="H5" s="1"/>
       <c r="I5" s="1"/>
       <c r="J5" s="1"/>
       <c r="K5" s="1"/>
       <c r="L5" s="1"/>
       <c r="M5" s="1"/>
-      <c r="N5" s="1"/>
+      <c r="N5" s="4"/>
       <c r="O5" s="5"/>
-      <c r="P5" s="6"/>
-      <c r="Q5" s="6"/>
-      <c r="R5" s="6"/>
-      <c r="S5" s="11"/>
-      <c r="T5" s="11"/>
-      <c r="U5" s="11"/>
-      <c r="V5" s="11"/>
-      <c r="W5" s="11"/>
-      <c r="X5" s="11"/>
+      <c r="P5" s="5"/>
+      <c r="Q5" s="5"/>
+      <c r="R5" s="10"/>
+      <c r="S5" s="10"/>
+      <c r="T5" s="10"/>
+      <c r="U5" s="10"/>
+      <c r="V5" s="10"/>
+      <c r="W5" s="10"/>
+      <c r="X5" s="10"/>
     </row>
-    <row r="6" spans="1:24" s="10" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="14" t="s">
+    <row r="6" spans="1:24" s="9" customFormat="1" ht="24" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A6" s="13" t="s">
         <v>3</v>
       </c>
-      <c r="B6" s="14"/>
-      <c r="C6" s="14"/>
-      <c r="D6" s="14"/>
-      <c r="E6" s="14"/>
-      <c r="F6" s="14"/>
-      <c r="G6" s="12" t="s">
+      <c r="B6" s="13"/>
+      <c r="C6" s="13"/>
+      <c r="D6" s="13"/>
+      <c r="E6" s="13"/>
+      <c r="F6" s="11" t="s">
         <v>27</v>
       </c>
-      <c r="H6" s="12" t="s">
+      <c r="G6" s="11" t="s">
         <v>28</v>
       </c>
-      <c r="I6" s="12" t="s">
+      <c r="H6" s="11" t="s">
         <v>29</v>
       </c>
-      <c r="J6" s="12" t="s">
+      <c r="I6" s="11" t="s">
         <v>30</v>
       </c>
-      <c r="K6" s="12" t="s">
+      <c r="J6" s="11" t="s">
         <v>31</v>
       </c>
-      <c r="L6" s="3" t="s">
+      <c r="K6" s="11" t="s">
         <v>32</v>
       </c>
-      <c r="M6" s="3" t="s">
+      <c r="L6" s="11" t="s">
         <v>33</v>
       </c>
-      <c r="N6" s="3" t="s">
+      <c r="M6" s="11" t="s">
         <v>34</v>
       </c>
-      <c r="O6" s="3" t="s">
+      <c r="N6" s="11" t="s">
         <v>35</v>
       </c>
-      <c r="P6" s="3" t="s">
+      <c r="O6" s="11" t="s">
         <v>36</v>
       </c>
-      <c r="Q6" s="3" t="s">
+      <c r="P6" s="11" t="s">
         <v>37</v>
       </c>
-      <c r="R6" s="3" t="s">
+      <c r="Q6" s="11" t="s">
         <v>38</v>
       </c>
-      <c r="S6" s="11"/>
-      <c r="T6" s="15"/>
-      <c r="U6" s="15"/>
-      <c r="V6" s="15"/>
-      <c r="W6" s="15"/>
-      <c r="X6" s="15"/>
+      <c r="R6" s="10"/>
+      <c r="S6" s="10"/>
+      <c r="T6" s="14"/>
+      <c r="U6" s="14"/>
+      <c r="V6" s="14"/>
+      <c r="W6" s="14"/>
+      <c r="X6" s="14"/>
     </row>
-    <row r="7" spans="1:24" s="10" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="14"/>
-      <c r="B7" s="14"/>
-      <c r="C7" s="14"/>
-      <c r="D7" s="14"/>
-      <c r="E7" s="14"/>
-      <c r="F7" s="14"/>
-      <c r="G7" s="12">
+    <row r="7" spans="1:24" s="9" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A7" s="13"/>
+      <c r="B7" s="13"/>
+      <c r="C7" s="13"/>
+      <c r="D7" s="13"/>
+      <c r="E7" s="13"/>
+      <c r="F7" s="11" t="s">
+        <v>54</v>
+      </c>
+      <c r="G7" s="11" t="s">
+        <v>54</v>
+      </c>
+      <c r="H7" s="11" t="s">
+        <v>54</v>
+      </c>
+      <c r="I7" s="11" t="s">
+        <v>54</v>
+      </c>
+      <c r="J7" s="11" t="s">
+        <v>54</v>
+      </c>
+      <c r="K7" s="11" t="s">
+        <v>54</v>
+      </c>
+      <c r="L7" s="11" t="s">
+        <v>54</v>
+      </c>
+      <c r="M7" s="11" t="s">
+        <v>54</v>
+      </c>
+      <c r="N7" s="1" t="s">
+        <v>54</v>
+      </c>
+      <c r="O7" s="11" t="s">
+        <v>54</v>
+      </c>
+      <c r="P7" s="11" t="s">
+        <v>54</v>
+      </c>
+      <c r="Q7" s="11" t="s">
+        <v>54</v>
+      </c>
+      <c r="R7" s="10"/>
+      <c r="S7" s="10"/>
+      <c r="T7" s="14"/>
+      <c r="U7" s="14"/>
+      <c r="V7" s="14"/>
+      <c r="W7" s="14"/>
+      <c r="X7" s="14"/>
+    </row>
+    <row r="8" spans="1:24" s="9" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A8" s="13" t="s">
+        <v>4</v>
+      </c>
+      <c r="B8" s="13"/>
+      <c r="C8" s="13"/>
+      <c r="D8" s="13"/>
+      <c r="E8" s="13"/>
+      <c r="F8" s="12">
         <v>0</v>
       </c>
-      <c r="H7" s="12">
-        <v>0</v>
-      </c>
-      <c r="I7" s="12">
-        <v>0</v>
-      </c>
-      <c r="J7" s="12">
-        <v>0</v>
-      </c>
-      <c r="K7" s="12">
-        <v>0</v>
-      </c>
-      <c r="L7" s="3"/>
-      <c r="M7" s="3"/>
-      <c r="N7" s="3"/>
-      <c r="O7" s="3"/>
-      <c r="P7" s="3"/>
-      <c r="Q7" s="3"/>
-      <c r="R7" s="3"/>
-      <c r="S7" s="11"/>
-      <c r="T7" s="15"/>
-      <c r="U7" s="15"/>
-      <c r="V7" s="15"/>
-      <c r="W7" s="15"/>
-      <c r="X7" s="15"/>
+      <c r="G8" s="2"/>
+      <c r="H8" s="3"/>
+      <c r="I8" s="3"/>
+      <c r="J8" s="3"/>
+      <c r="K8" s="3"/>
+      <c r="L8" s="3"/>
+      <c r="M8" s="3"/>
+      <c r="N8" s="10"/>
+      <c r="O8" s="10"/>
+      <c r="P8" s="10"/>
+      <c r="Q8" s="10"/>
+      <c r="R8" s="10"/>
+      <c r="S8" s="10"/>
+      <c r="T8" s="10"/>
+      <c r="U8" s="10"/>
+      <c r="V8" s="10"/>
+      <c r="W8" s="10"/>
+      <c r="X8" s="10"/>
     </row>
-    <row r="8" spans="1:24" s="10" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A8" s="14" t="s">
-        <v>4</v>
-      </c>
-      <c r="B8" s="14"/>
-      <c r="C8" s="14"/>
-      <c r="D8" s="14"/>
-      <c r="E8" s="14"/>
-      <c r="F8" s="14"/>
-      <c r="G8" s="13">
-        <v>0</v>
-      </c>
-      <c r="H8" s="2"/>
-      <c r="I8" s="4"/>
-      <c r="J8" s="4"/>
-      <c r="K8" s="4"/>
-      <c r="L8" s="4"/>
-      <c r="M8" s="4"/>
-      <c r="N8" s="4"/>
-      <c r="O8" s="11"/>
-      <c r="P8" s="11"/>
-      <c r="Q8" s="11"/>
-      <c r="R8" s="11"/>
-      <c r="S8" s="11"/>
-      <c r="T8" s="11"/>
-      <c r="U8" s="11"/>
-      <c r="V8" s="11"/>
-      <c r="W8" s="11"/>
-      <c r="X8" s="11"/>
-    </row>
-    <row r="9" spans="1:24" s="10" customFormat="1" ht="31.5" x14ac:dyDescent="0.2">
-      <c r="A9" s="7" t="s">
+    <row r="9" spans="1:24" s="9" customFormat="1" ht="31.5" x14ac:dyDescent="0.2">
+      <c r="A9" s="6" t="s">
         <v>5</v>
       </c>
-      <c r="B9" s="7" t="s">
+      <c r="B9" s="6" t="s">
+        <v>46</v>
+      </c>
+      <c r="C9" s="6" t="s">
+        <v>48</v>
+      </c>
+      <c r="D9" s="6" t="s">
         <v>47</v>
       </c>
-      <c r="C9" s="7" t="s">
-        <v>49</v>
-      </c>
-      <c r="D9" s="7" t="s">
-        <v>48</v>
-      </c>
-      <c r="E9" s="7" t="s">
+      <c r="E9" s="6" t="s">
         <v>6</v>
       </c>
-      <c r="F9" s="7" t="s">
+      <c r="F9" s="6" t="s">
         <v>7</v>
       </c>
-      <c r="G9" s="8" t="s">
+      <c r="G9" s="7" t="s">
         <v>8</v>
       </c>
-      <c r="H9" s="9" t="s">
+      <c r="H9" s="8" t="s">
         <v>10</v>
       </c>
-      <c r="I9" s="9" t="s">
+      <c r="I9" s="8" t="s">
         <v>11</v>
       </c>
-      <c r="J9" s="9" t="s">
+      <c r="J9" s="8" t="s">
         <v>12</v>
       </c>
-      <c r="K9" s="9" t="s">
+      <c r="K9" s="8" t="s">
         <v>13</v>
       </c>
-      <c r="L9" s="9" t="s">
+      <c r="L9" s="8" t="s">
         <v>14</v>
       </c>
-      <c r="M9" s="9" t="s">
+      <c r="M9" s="8" t="s">
         <v>15</v>
       </c>
-      <c r="N9" s="9" t="s">
+      <c r="N9" s="8" t="s">
         <v>16</v>
       </c>
-      <c r="O9" s="9" t="s">
+      <c r="O9" s="8" t="s">
         <v>17</v>
       </c>
-      <c r="P9" s="9" t="s">
+      <c r="P9" s="8" t="s">
         <v>18</v>
       </c>
-      <c r="Q9" s="9" t="s">
+      <c r="Q9" s="8" t="s">
         <v>19</v>
       </c>
-      <c r="R9" s="9" t="s">
+      <c r="R9" s="8" t="s">
         <v>20</v>
       </c>
-      <c r="S9" s="9" t="s">
+      <c r="S9" s="8" t="s">
         <v>21</v>
       </c>
-      <c r="T9" s="9" t="s">
+      <c r="T9" s="8" t="s">
         <v>22</v>
       </c>
-      <c r="U9" s="9" t="s">
+      <c r="U9" s="8" t="s">
         <v>23</v>
       </c>
-      <c r="V9" s="8" t="s">
+      <c r="V9" s="7" t="s">
         <v>24</v>
       </c>
-      <c r="W9" s="8" t="s">
+      <c r="W9" s="7" t="s">
         <v>9</v>
       </c>
-      <c r="X9" s="8" t="s">
+      <c r="X9" s="7" t="s">
         <v>25</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="12">
-    <mergeCell ref="A5:F5"/>
-    <mergeCell ref="A8:F8"/>
+    <mergeCell ref="A6:E7"/>
+    <mergeCell ref="A8:E8"/>
     <mergeCell ref="T6:T7"/>
     <mergeCell ref="A1:X1"/>
-    <mergeCell ref="A2:F2"/>
-    <mergeCell ref="A4:F4"/>
-    <mergeCell ref="A6:F7"/>
     <mergeCell ref="W6:W7"/>
     <mergeCell ref="X6:X7"/>
     <mergeCell ref="U6:U7"/>
     <mergeCell ref="V6:V7"/>
-    <mergeCell ref="A3:F3"/>
+    <mergeCell ref="A2:E2"/>
+    <mergeCell ref="A3:E3"/>
+    <mergeCell ref="A4:E4"/>
+    <mergeCell ref="A5:E5"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>